<commit_message>
Enhance header normalization and update productivity export functionality
- Introduced HEADER_ALIASES in `erection_compiled_to_daily_new.py` to improve header matching for data normalization.
- Refactored EXPECTED_HEADER_KEYS to utilize aliases, enhancing the robustness of header detection.
- Updated `export_erection_summary.py` to include new command-line arguments for date range exports and improved project PCH mapping handling.
- Enhanced `export_kv_productivity_summary.py` with start and end month options for continuous range summarization.
- Deleted outdated Excel files to streamline the project directory.
</commit_message>
<xml_diff>
--- a/Raw Data/Email_config.xlsx
+++ b/Raw Data/Email_config.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C7BE41-AAE3-4DEB-A656-6A35DBFACFA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842B5697-1F58-40E1-9194-0E66D7680659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="65">
   <si>
     <t>Name</t>
   </si>
@@ -69,9 +80,6 @@
     <t>Santosh Kumar</t>
   </si>
   <si>
-    <t>Partha Pratim Pal &lt;palp04@kecrpg.com&gt;</t>
-  </si>
-  <si>
     <t>Work Progress of 765 kV D/C Hexa Beawar-Mandsaur T/L</t>
   </si>
   <si>
@@ -99,9 +107,6 @@
     <t>Janvendra Kumar</t>
   </si>
   <si>
-    <t>Sanjib Kumar Samantaray &lt;samantaraysk@kecrpg.com&gt;</t>
-  </si>
-  <si>
     <t>Raghav Ranjan</t>
   </si>
   <si>
@@ -111,9 +116,6 @@
     <t>sharmap07@KECRPG.COM</t>
   </si>
   <si>
-    <t>S Ajith JayaSurya &lt;jayaSuryaa@kecrpg.com&gt;</t>
-  </si>
-  <si>
     <t>DPR _765KV D/C Koppal II (PS) -Raichur TL Part-1</t>
   </si>
   <si>
@@ -121,6 +123,114 @@
   </si>
   <si>
     <t>DPR -BMTL</t>
+  </si>
+  <si>
+    <t>Santosh Pandey</t>
+  </si>
+  <si>
+    <t>Amartya Sarkar</t>
+  </si>
+  <si>
+    <t>Harshit Kumar</t>
+  </si>
+  <si>
+    <t>M Aditya Narsimha</t>
+  </si>
+  <si>
+    <t>Nishant Giri</t>
+  </si>
+  <si>
+    <t>Daily Progress Report, Visual Chart &amp; Hindrance Register - Bikaner-IV PS - SiwSuraj Kumar &lt;kumarsu@kecrpg.com&gt;ani 765kV D/C 2nd Tr. Line (Part-01) TA-512</t>
+  </si>
+  <si>
+    <t>Saurabh Katiyar</t>
+  </si>
+  <si>
+    <t>katiyars@kecrpg.com</t>
+  </si>
+  <si>
+    <t>DPR TB401  Sterlite 765KV F3BTL 20.12.25.</t>
+  </si>
+  <si>
+    <t>pandeysa@kecrpg.com</t>
+  </si>
+  <si>
+    <t>DPR of TB 507 400kV D/C Fatehgarh IV - Bhinmal(PG) Transmission Line</t>
+  </si>
+  <si>
+    <t>sarkara1@kecrpg.com</t>
+  </si>
+  <si>
+    <t>kumarh02@kecrpg.com</t>
+  </si>
+  <si>
+    <t>kumarm42@kecrpg.com</t>
+  </si>
+  <si>
+    <t>DPR - Ratle Kiru Power Transmission Ltd (TB-605)  - Dt: 21-12-2025</t>
+  </si>
+  <si>
+    <t>TL-04 765kV VNTL DPR</t>
+  </si>
+  <si>
+    <t>girin@kecrpg.com</t>
+  </si>
+  <si>
+    <t>Possible_Attachement_Name</t>
+  </si>
+  <si>
+    <t>Partha Pratim Pal</t>
+  </si>
+  <si>
+    <t>S Ajith JayaSurya</t>
+  </si>
+  <si>
+    <t>Sanjib Kumar Samantaray</t>
+  </si>
+  <si>
+    <t>DPR_765 KV DC BIKANER IV PS TO SIWANI II</t>
+  </si>
+  <si>
+    <t>Suraj Kumar</t>
+  </si>
+  <si>
+    <t>kumarsu@kecrpg.com</t>
+  </si>
+  <si>
+    <t>DPR of Project-TA-509</t>
+  </si>
+  <si>
+    <t>Visual Chart TA 509</t>
+  </si>
+  <si>
+    <t>kumarp72@kecrpg.com</t>
+  </si>
+  <si>
+    <t>Prashant Kumar</t>
+  </si>
+  <si>
+    <t>DPR || 400KV Siwani-Fatehabad TL &amp; 400 KV Siwani-Patran TL</t>
+  </si>
+  <si>
+    <t>Project_Code</t>
+  </si>
+  <si>
+    <t>TA 509</t>
+  </si>
+  <si>
+    <t>TA 512</t>
+  </si>
+  <si>
+    <t>TA 513</t>
+  </si>
+  <si>
+    <t>TA 414</t>
+  </si>
+  <si>
+    <t>VNTL KEC DPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPR-T513 </t>
   </si>
 </sst>
 </file>
@@ -438,10 +548,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="48.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.453125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -451,74 +566,80 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
         <v>4</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>6</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
         <v>7</v>
       </c>
       <c r="C6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -526,21 +647,21 @@
         <v>9</v>
       </c>
       <c r="C8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
         <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -548,15 +669,142 @@
         <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C16" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
+        <v>44</v>
+      </c>
+      <c r="D18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>56</v>
+      </c>
+      <c r="B19" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" t="s">
+        <v>57</v>
+      </c>
+      <c r="D19" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Patch/dpr sheet config logic (#4)
* Auto pipeline update 2026-02-24 12:09:46

* Auto pipeline update 2026-02-24 16:07:51

* Auto pipeline update 2026-02-25 11:38:21

* Auto pipeline update 2026-02-25 12:09:15

* Auto pipeline update 2026-02-25 12:09:38

* Auto pipeline update 2026-02-25 16:10:18

* Auto pipeline update 2026-02-25 16:11:05

* Fix: Sheet config logic

* Auto pipeline update 2026-02-26 11:38:42

* Auto pipeline update 2026-02-26 12:10:41

* Auto pipeline update 2026-02-26 12:10:52

* Auto pipeline update 2026-02-26 16:08:51

* Auto pipeline update 2026-02-27 11:41:23

* Auto pipeline update 2026-02-27 11:41:58

* Fix: Sheet config logic

* Auto pipeline update 2026-02-27 12:13:32

* Auto pipeline update 2026-02-27 12:14:20
</commit_message>
<xml_diff>
--- a/Raw Data/Email_config.xlsx
+++ b/Raw Data/Email_config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842B5697-1F58-40E1-9194-0E66D7680659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F22891-5597-447E-BC4F-3DE043FF928D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
   <si>
     <t>Name</t>
   </si>
@@ -231,6 +231,33 @@
   </si>
   <si>
     <t xml:space="preserve">DPR-T513 </t>
+  </si>
+  <si>
+    <t>Siddhesh Bhoyar</t>
+  </si>
+  <si>
+    <t>bhoyars@kecrpg.com</t>
+  </si>
+  <si>
+    <t>DPR of Package TL02 for 765kV D/C Kurnool IV – Bidar Line Part-II</t>
+  </si>
+  <si>
+    <t>TA 601</t>
+  </si>
+  <si>
+    <t>TL-02_Kurnool_IV-Bidar_DPR</t>
+  </si>
+  <si>
+    <t>TB401 : Daily Progress Report for 765KV DC Fategarh III to Beawar (2nd) TL (PKG-G)</t>
+  </si>
+  <si>
+    <t>sainij@kecrpg.com</t>
+  </si>
+  <si>
+    <t>Saini Jitendra</t>
+  </si>
+  <si>
+    <t>TB 401</t>
   </si>
 </sst>
 </file>
@@ -548,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48.26953125" bestFit="1" customWidth="1"/>
@@ -807,6 +834,37 @@
         <v>61</v>
       </c>
     </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D20" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto pipeline update 2026-03-03 11:39:52
</commit_message>
<xml_diff>
--- a/Raw Data/Email_config.xlsx
+++ b/Raw Data/Email_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F22891-5597-447E-BC4F-3DE043FF928D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB13EBBE-CDC5-4A06-A3D1-004714CE0AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="78">
   <si>
     <t>Name</t>
   </si>
@@ -258,6 +258,18 @@
   </si>
   <si>
     <t>TB 401</t>
+  </si>
+  <si>
+    <t>Copy of DPR TB 507 765 kV LILO FTH-III_BW_at_FTH-IV TL TS; TB 507 - DPR -TB 507_Sindhari</t>
+  </si>
+  <si>
+    <t>Line_Name</t>
+  </si>
+  <si>
+    <t>LILO; MAIN</t>
+  </si>
+  <si>
+    <t>TB 507</t>
   </si>
 </sst>
 </file>
@@ -575,7 +587,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48.26953125" bestFit="1" customWidth="1"/>
@@ -583,7 +595,7 @@
     <col min="3" max="3" width="53.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -597,10 +609,13 @@
         <v>46</v>
       </c>
       <c r="E1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F1" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>47</v>
       </c>
@@ -611,7 +626,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -622,7 +637,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -633,7 +648,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -644,7 +659,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>48</v>
       </c>
@@ -655,7 +670,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -666,7 +681,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -677,7 +692,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -688,7 +703,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -699,7 +714,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -712,11 +727,11 @@
       <c r="D11" t="s">
         <v>54</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>51</v>
       </c>
@@ -729,11 +744,11 @@
       <c r="D12" t="s">
         <v>50</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>35</v>
       </c>
@@ -746,11 +761,11 @@
       <c r="D13" t="s">
         <v>50</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>29</v>
       </c>
@@ -761,7 +776,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -771,8 +786,17 @@
       <c r="C15" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="D15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" t="s">
+        <v>76</v>
+      </c>
+      <c r="F15" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -785,11 +809,11 @@
       <c r="D16" t="s">
         <v>64</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>32</v>
       </c>
@@ -800,7 +824,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -813,11 +837,11 @@
       <c r="D18" t="s">
         <v>63</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>56</v>
       </c>
@@ -830,11 +854,11 @@
       <c r="D19" t="s">
         <v>64</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>65</v>
       </c>
@@ -847,11 +871,11 @@
       <c r="D20" t="s">
         <v>69</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -861,7 +885,7 @@
       <c r="C21" t="s">
         <v>70</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>73</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto pipeline update 2026-03-10 10:38:04
</commit_message>
<xml_diff>
--- a/Raw Data/Email_config.xlsx
+++ b/Raw Data/Email_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB13EBBE-CDC5-4A06-A3D1-004714CE0AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{329BA73F-CCE9-42A6-9CE7-80041A73B550}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="83">
   <si>
     <t>Name</t>
   </si>
@@ -270,6 +270,21 @@
   </si>
   <si>
     <t>TB 507</t>
+  </si>
+  <si>
+    <t>shuklap05@KECRPG.COM</t>
+  </si>
+  <si>
+    <t>Prashun Shukla</t>
+  </si>
+  <si>
+    <t>220kV and 132kV Neemuch TL DPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPR of 220kV and 132kV Neemuch Chanderiya TL </t>
+  </si>
+  <si>
+    <t>Test 000</t>
   </si>
 </sst>
 </file>
@@ -587,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48.26953125" bestFit="1" customWidth="1"/>
@@ -889,6 +904,23 @@
         <v>73</v>
       </c>
     </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>79</v>
+      </c>
+      <c r="B22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" t="s">
+        <v>81</v>
+      </c>
+      <c r="D22" t="s">
+        <v>80</v>
+      </c>
+      <c r="F22" t="s">
+        <v>82</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto pipeline update 2026-03-11 11:36:41
</commit_message>
<xml_diff>
--- a/Raw Data/Email_config.xlsx
+++ b/Raw Data/Email_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E84BE010-2233-494B-8F4F-58EE3815DF8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B684C76-72A6-42FE-8D69-D853C0563571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -284,7 +284,7 @@
     <t xml:space="preserve">DPR of 220kV and 132kV Neemuch Chanderiya TL </t>
   </si>
   <si>
-    <t>Test 000</t>
+    <t>TB 501</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Auto pipeline update 2026-07-07 10:49:41
</commit_message>
<xml_diff>
--- a/Raw Data/Email_config.xlsx
+++ b/Raw Data/Email_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E02E50E-A543-4FE4-B343-8127DF8B39A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B11AC19-0045-4B8D-B88C-F37556E47DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="133">
   <si>
     <t>Name</t>
   </si>
@@ -429,6 +429,12 @@
   </si>
   <si>
     <t>TB 412</t>
+  </si>
+  <si>
+    <t>dass33@KECRPG.COM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sony Das </t>
   </si>
 </sst>
 </file>
@@ -757,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48.26953125" bestFit="1" customWidth="1"/>
@@ -1269,9 +1275,27 @@
         <v>130</v>
       </c>
     </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>132</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C34" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" t="s">
+        <v>61</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B24" r:id="rId1" xr:uid="{4A677AC9-19C7-45A7-B3EB-DC8C0C43E6EB}"/>
+    <hyperlink ref="B34" r:id="rId2" xr:uid="{61B8A444-F57E-4F33-A7D9-FD2ACD1D75B8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto pipeline update 2026-08-11 12:19:18
</commit_message>
<xml_diff>
--- a/Raw Data/Email_config.xlsx
+++ b/Raw Data/Email_config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B11AC19-0045-4B8D-B88C-F37556E47DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B537AFD1-1B7E-4CA5-930F-8D18C9E7C87E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="138">
   <si>
     <t>Name</t>
   </si>
@@ -435,6 +435,21 @@
   </si>
   <si>
     <t xml:space="preserve">Sony Das </t>
+  </si>
+  <si>
+    <t>Jigar Karena</t>
+  </si>
+  <si>
+    <t>DPR - Ratle Kiru Power Transmission Ltd (TB-605)</t>
+  </si>
+  <si>
+    <t>karenaj@KECRPG.COM</t>
+  </si>
+  <si>
+    <t>DPR TB-605 RKPTL</t>
+  </si>
+  <si>
+    <t>TB 605</t>
   </si>
 </sst>
 </file>
@@ -763,7 +778,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="48.26953125" bestFit="1" customWidth="1"/>
@@ -1292,6 +1307,23 @@
         <v>61</v>
       </c>
     </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" t="s">
+        <v>135</v>
+      </c>
+      <c r="C35" t="s">
+        <v>134</v>
+      </c>
+      <c r="D35" t="s">
+        <v>136</v>
+      </c>
+      <c r="F35" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B24" r:id="rId1" xr:uid="{4A677AC9-19C7-45A7-B3EB-DC8C0C43E6EB}"/>

</xml_diff>